<commit_message>
Normalize match schema and date format
Updates the World Cup dataset to a machine-friendly structure by converting `date` values to `YYYY-MM-DD`, replacing `score` with numeric `home_score`/`away_score`, and removing the derived `result` field. `xls-to-json.py` now normalizes dates during export, and the JSON/XLSX data were regenerated with these schema changes (including updated match entries). Also adds `sample.py` to print formatted match results from the new JSON shape.
</commit_message>
<xml_diff>
--- a/worldcup26.xlsx
+++ b/worldcup26.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tatam\Projects\myproj\WorldCup26\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tatam\Projects\myproj\WorldCup2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D77C22F-C2AE-487E-A4FF-0F305139DD1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA52C0B3-30D2-4C79-8414-3BDB23A5615E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2955" yWindow="75" windowWidth="33540" windowHeight="20010" xr2:uid="{B5805A21-8289-4030-9022-D7B0EEB9AFF6}"/>
+    <workbookView xWindow="3345" yWindow="645" windowWidth="33540" windowHeight="20010" xr2:uid="{B5805A21-8289-4030-9022-D7B0EEB9AFF6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="114">
   <si>
     <t>グループA</t>
   </si>
@@ -282,21 +282,6 @@
     <t>コロンビア</t>
   </si>
   <si>
-    <t>0-1</t>
-  </si>
-  <si>
-    <t>0-0</t>
-  </si>
-  <si>
-    <t>0-4</t>
-  </si>
-  <si>
-    <t>0-3</t>
-  </si>
-  <si>
-    <t>0-2</t>
-  </si>
-  <si>
     <t>PK:3-4</t>
   </si>
   <si>
@@ -312,205 +297,7 @@
     <t>PK戦:5-4</t>
   </si>
   <si>
-    <t>2-0</t>
-  </si>
-  <si>
     <t/>
-  </si>
-  <si>
-    <t>2-1</t>
-  </si>
-  <si>
-    <t>1-1</t>
-  </si>
-  <si>
-    <t>4-1</t>
-  </si>
-  <si>
-    <t>1-0</t>
-  </si>
-  <si>
-    <t>7-1</t>
-  </si>
-  <si>
-    <t>2-2</t>
-  </si>
-  <si>
-    <t>5-1</t>
-  </si>
-  <si>
-    <t>3-1</t>
-  </si>
-  <si>
-    <t>1-4</t>
-  </si>
-  <si>
-    <t>3-0</t>
-  </si>
-  <si>
-    <t>4-2</t>
-  </si>
-  <si>
-    <t>1-3</t>
-  </si>
-  <si>
-    <t>6-0</t>
-  </si>
-  <si>
-    <t>4-0</t>
-  </si>
-  <si>
-    <t>3-2</t>
-  </si>
-  <si>
-    <t>1-2</t>
-  </si>
-  <si>
-    <t>5-0</t>
-  </si>
-  <si>
-    <t>1-5</t>
-  </si>
-  <si>
-    <t>3-3</t>
-  </si>
-  <si>
-    <t>2-3</t>
-  </si>
-  <si>
-    <t>4-6</t>
-  </si>
-  <si>
-    <t>2026年6⽉11⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉12⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉13⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉14⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉15⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉16⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉17⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉19⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉20⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉21⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉22⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉23⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉24⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉25⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉26⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉27⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉28⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉29⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年6⽉30⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年7⽉1⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年7⽉2⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年7⽉3⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年7⽉4⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年7⽉5⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年7⽉6⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年7⽉7⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年7⽉9⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年7⽉10⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年7⽉11⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年7月14日</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年7⽉15⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年7⽉18⽇</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
-    <t>2026年7⽉19⽇</t>
-    <phoneticPr fontId="3"/>
   </si>
   <si>
     <t>date</t>
@@ -525,18 +312,10 @@
     <phoneticPr fontId="3"/>
   </si>
   <si>
-    <t>score</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
     <t>notes</t>
     <phoneticPr fontId="3"/>
   </si>
   <si>
-    <t>result</t>
-    <phoneticPr fontId="3"/>
-  </si>
-  <si>
     <t>group</t>
     <phoneticPr fontId="3"/>
   </si>
@@ -618,6 +397,22 @@
   </si>
   <si>
     <t xml:space="preserve"> ロサンゼルス・スタジアム</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>home_score</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>away_score</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>スペイン</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>ベルギー</t>
     <phoneticPr fontId="3"/>
   </si>
 </sst>
@@ -625,6 +420,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -687,26 +485,18 @@
       <charset val="128"/>
     </font>
     <font>
-      <b/>
       <sz val="7"/>
-      <color rgb="FFFFFFFF"/>
       <name val="メイリオ"/>
       <family val="3"/>
       <charset val="128"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -726,7 +516,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -734,19 +524,237 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="ハイパーリンク" xfId="1" builtinId="8"/>
     <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="10">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="7"/>
+        <color rgb="FF0369C7"/>
+        <name val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="7"/>
+        <color auto="1"/>
+        <name val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <name val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="7"/>
+        <color rgb="FF03122B"/>
+        <name val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="7"/>
+        <color rgb="FF000000"/>
+        <name val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="7"/>
+        <color rgb="FF0369C7"/>
+        <name val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="7"/>
+        <color rgb="FF0369C7"/>
+        <name val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="7"/>
+        <color rgb="FF0369C7"/>
+        <name val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="7"/>
+        <color rgb="FF0369C7"/>
+        <name val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="7"/>
+        <color rgb="FF03122B"/>
+        <name val="メイリオ"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd;@"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -757,6 +765,24 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{92835F56-59CC-45E0-9CD6-BF3448062B44}" name="テーブル1" displayName="テーブル1" ref="A1:I105" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:I105" xr:uid="{92835F56-59CC-45E0-9CD6-BF3448062B44}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{ECF33BFB-21A5-4458-9220-8C22484CBDBE}" name="date" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{F3E1F2D8-1B73-4BAD-84CA-9DA0B4D3914D}" name="home" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{39B24F56-D0D4-4C89-B477-B850C237B0DF}" name="home_score" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{0C7DF10C-8C15-48EC-BABB-D1C6C9E6DDA9}" name="away" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{32117AF7-FE83-4DBB-98AE-A5726BCFDC4F}" name="away_score" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{A78DFA17-4341-4B39-B545-715DEE3E5BCF}" name="notes" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{2D0BC01B-0B5C-4AFA-B2C9-C6887D8CA2B5}" name="group" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{1DCEADB5-2DE2-4B12-A7BF-BD9D4AA3D095}" name="stage" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{E740C332-3DD1-4F9F-854F-DB597E5E9B26}" name="studium" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1079,66 +1105,64 @@
   <dimension ref="A1:I105"/>
   <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="15.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.875" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9" style="3"/>
+    <col min="1" max="1" width="9.375" style="8" customWidth="1"/>
+    <col min="2" max="2" width="15.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.875" style="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.625" style="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.25" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.25" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="27.25" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>153</v>
+    <row r="1" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
-        <v>112</v>
+      <c r="A2" s="9">
+        <v>46184</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="14">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F2" s="1" t="str">
-        <f>_xlfn.LET(_xlpm.s,D2,_xlpm.hs,--_xlfn.TEXTBEFORE(_xlpm.s,"-"),_xlpm.as,--_xlfn.TEXTAFTER(_xlpm.s,"-"),IF(_xlpm.hs&gt;_xlpm.as,B2,IF(_xlpm.hs&lt;_xlpm.as,C2,"引き分け")))</f>
-        <v>メキシコ</v>
-      </c>
+      <c r="E2" s="14">
+        <v>0</v>
+      </c>
+      <c r="F2" s="5"/>
       <c r="G2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1146,28 +1170,27 @@
         <v>1</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>154</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
-        <v>112</v>
+      <c r="A3" s="9">
+        <v>46184</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="14">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F3" s="1" t="str">
-        <f t="shared" ref="F3:F66" si="0">_xlfn.LET(_xlpm.s,D3,_xlpm.hs,--_xlfn.TEXTBEFORE(_xlpm.s,"-"),_xlpm.as,--_xlfn.TEXTAFTER(_xlpm.s,"-"),IF(_xlpm.hs&gt;_xlpm.as,B3,IF(_xlpm.hs&lt;_xlpm.as,C3,"引き分け")))</f>
-        <v>韓国</v>
+      <c r="E3" s="14">
+        <v>1</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>0</v>
@@ -1176,28 +1199,27 @@
         <v>1</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>155</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
-        <v>113</v>
+      <c r="A4" s="9">
+        <v>46185</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="14">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F4" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E4" s="14">
+        <v>1</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>2</v>
@@ -1206,28 +1228,27 @@
         <v>1</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>156</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
-        <v>113</v>
+      <c r="A5" s="9">
+        <v>46185</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="14">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F5" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>アメリカ</v>
+      <c r="E5" s="14">
+        <v>1</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>3</v>
@@ -1236,28 +1257,27 @@
         <v>1</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>157</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
-        <v>114</v>
+      <c r="A6" s="9">
+        <v>46186</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="14">
+        <v>0</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F6" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>スコットランド</v>
+      <c r="E6" s="14">
+        <v>1</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>4</v>
@@ -1266,28 +1286,27 @@
         <v>1</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>158</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
-        <v>114</v>
+      <c r="A7" s="9">
+        <v>46186</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="14">
+        <v>2</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F7" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>オーストラリア</v>
+      <c r="E7" s="14">
+        <v>0</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>5</v>
@@ -1296,28 +1315,27 @@
         <v>1</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>159</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
-        <v>114</v>
+      <c r="A8" s="9">
+        <v>46186</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="14">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F8" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E8" s="14">
+        <v>1</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>6</v>
@@ -1326,28 +1344,27 @@
         <v>1</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>160</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
-        <v>114</v>
+      <c r="A9" s="9">
+        <v>46186</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="14">
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F9" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E9" s="14">
+        <v>1</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>2</v>
@@ -1356,28 +1373,27 @@
         <v>1</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>161</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
-        <v>115</v>
+      <c r="A10" s="10">
+        <v>46187</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="14">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F10" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>コートジボワール</v>
+      <c r="E10" s="14">
+        <v>0</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>7</v>
@@ -1386,28 +1402,27 @@
         <v>1</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>162</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
-        <v>115</v>
+      <c r="A11" s="10">
+        <v>46187</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="14">
+        <v>7</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F11" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>ドイツ</v>
+      <c r="E11" s="14">
+        <v>1</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>7</v>
@@ -1416,28 +1431,27 @@
         <v>1</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>163</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
-        <v>115</v>
+      <c r="A12" s="10">
+        <v>46187</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="14">
+        <v>2</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F12" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E12" s="14">
+        <v>2</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>8</v>
@@ -1446,28 +1460,27 @@
         <v>1</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>164</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
-        <v>115</v>
+      <c r="A13" s="10">
+        <v>46187</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="14">
+        <v>5</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D13" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F13" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>スウェーデン</v>
+      <c r="E13" s="14">
+        <v>1</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>9</v>
@@ -1476,28 +1489,27 @@
         <v>1</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>165</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="9" t="s">
-        <v>116</v>
+      <c r="A14" s="9">
+        <v>46188</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="14">
+        <v>0</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D14" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F14" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E14" s="14">
+        <v>0</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>10</v>
@@ -1506,28 +1518,27 @@
         <v>1</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>166</v>
+        <v>104</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
-        <v>116</v>
+      <c r="A15" s="9">
+        <v>46188</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="14">
+        <v>1</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F15" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E15" s="14">
+        <v>1</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>10</v>
@@ -1536,28 +1547,27 @@
         <v>1</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>167</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
-        <v>116</v>
+      <c r="A16" s="9">
+        <v>46188</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="14">
+        <v>2</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F16" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E16" s="14">
+        <v>2</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>11</v>
@@ -1566,28 +1576,27 @@
         <v>1</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>157</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="9" t="s">
-        <v>116</v>
+      <c r="A17" s="9">
+        <v>46188</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="14">
+        <v>1</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F17" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E17" s="14">
+        <v>1</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>12</v>
@@ -1596,28 +1605,27 @@
         <v>1</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>168</v>
+        <v>106</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="9" t="s">
-        <v>117</v>
+      <c r="A18" s="9">
+        <v>46189</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="14">
+        <v>3</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D18" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F18" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>フランス</v>
+      <c r="E18" s="14">
+        <v>1</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -1626,28 +1634,27 @@
         <v>1</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>169</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="9" t="s">
-        <v>117</v>
+      <c r="A19" s="9">
+        <v>46189</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="14">
+        <v>1</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D19" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F19" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>ノルウェー</v>
+      <c r="E19" s="14">
+        <v>4</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -1656,28 +1663,27 @@
         <v>1</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>158</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="9" t="s">
-        <v>117</v>
+      <c r="A20" s="9">
+        <v>46189</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="14">
+        <v>3</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D20" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F20" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>アルゼンチン</v>
+      <c r="E20" s="14">
+        <v>0</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>14</v>
@@ -1686,28 +1692,27 @@
         <v>1</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>170</v>
+        <v>108</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
-        <v>117</v>
+      <c r="A21" s="9">
+        <v>46189</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="14">
+        <v>3</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D21" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F21" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>オーストリア</v>
+      <c r="E21" s="14">
+        <v>1</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>15</v>
@@ -1716,28 +1721,27 @@
         <v>1</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>161</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="9" t="s">
-        <v>118</v>
+      <c r="A22" s="9">
+        <v>46190</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="14">
+        <v>1</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D22" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F22" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>ガーナ</v>
+      <c r="E22" s="14">
+        <v>0</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>16</v>
@@ -1746,28 +1750,27 @@
         <v>1</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>156</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="9" t="s">
-        <v>118</v>
+      <c r="A23" s="9">
+        <v>46190</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="14">
+        <v>4</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F23" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>イングランド</v>
+      <c r="E23" s="14">
+        <v>2</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>16</v>
@@ -1776,28 +1779,27 @@
         <v>1</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>164</v>
+        <v>102</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="9" t="s">
-        <v>118</v>
+      <c r="A24" s="9">
+        <v>46190</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" s="14">
+        <v>1</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D24" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F24" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E24" s="14">
+        <v>1</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>17</v>
@@ -1806,28 +1808,27 @@
         <v>1</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>163</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="9" t="s">
-        <v>118</v>
+      <c r="A25" s="9">
+        <v>46190</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" s="14">
+        <v>1</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D25" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F25" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>コロンビア</v>
+      <c r="E25" s="14">
+        <v>3</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>17</v>
@@ -1836,28 +1837,27 @@
         <v>1</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>154</v>
+        <v>92</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="9" t="s">
-        <v>118</v>
+      <c r="A26" s="9">
+        <v>46190</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="14">
+        <v>1</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D26" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F26" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E26" s="14">
+        <v>1</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>0</v>
@@ -1866,28 +1866,27 @@
         <v>1</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>166</v>
+        <v>104</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="9" t="s">
-        <v>118</v>
+      <c r="A27" s="9">
+        <v>46190</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" s="14">
+        <v>4</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D27" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F27" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>スイス</v>
+      <c r="E27" s="14">
+        <v>1</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>2</v>
@@ -1896,28 +1895,27 @@
         <v>1</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>157</v>
+        <v>95</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="9" t="s">
-        <v>118</v>
+      <c r="A28" s="9">
+        <v>46190</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" s="14">
+        <v>6</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D28" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F28" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>カナダ</v>
+      <c r="E28" s="14">
+        <v>0</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>2</v>
@@ -1926,28 +1924,27 @@
         <v>1</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>159</v>
+        <v>97</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" s="9" t="s">
-        <v>118</v>
+      <c r="A29" s="9">
+        <v>46190</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C29" s="14">
+        <v>1</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D29" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F29" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>メキシコ</v>
+      <c r="E29" s="14">
+        <v>0</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>0</v>
@@ -1956,28 +1953,27 @@
         <v>1</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>155</v>
+        <v>93</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="9" t="s">
-        <v>119</v>
+      <c r="A30" s="9">
+        <v>46192</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" s="14">
+        <v>2</v>
+      </c>
+      <c r="D30" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F30" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>アメリカ</v>
+      <c r="E30" s="14">
+        <v>0</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>3</v>
@@ -1986,28 +1982,27 @@
         <v>1</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>168</v>
+        <v>106</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" s="9" t="s">
-        <v>119</v>
+      <c r="A31" s="9">
+        <v>46192</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" s="14">
+        <v>3</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D31" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F31" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>ブラジル</v>
+      <c r="E31" s="14">
+        <v>0</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>6</v>
@@ -2016,28 +2011,27 @@
         <v>1</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>162</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="9" t="s">
-        <v>119</v>
+      <c r="A32" s="9">
+        <v>46192</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C32" s="14">
+        <v>0</v>
+      </c>
+      <c r="D32" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D32" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F32" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>モロッコ</v>
+      <c r="E32" s="14">
+        <v>1</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>6</v>
@@ -2046,28 +2040,27 @@
         <v>1</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>158</v>
+        <v>96</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" s="9" t="s">
-        <v>119</v>
+      <c r="A33" s="9">
+        <v>46192</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" s="14">
+        <v>0</v>
+      </c>
+      <c r="D33" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D33" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F33" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>パラグアイ</v>
+      <c r="E33" s="14">
+        <v>1</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>5</v>
@@ -2076,28 +2069,27 @@
         <v>1</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>161</v>
+        <v>99</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="7" t="s">
-        <v>120</v>
+      <c r="A34" s="10">
+        <v>46193</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" s="14">
+        <v>2</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D34" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F34" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>ドイツ</v>
+      <c r="E34" s="14">
+        <v>1</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>18</v>
@@ -2106,28 +2098,27 @@
         <v>1</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>156</v>
+        <v>94</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" s="7" t="s">
-        <v>120</v>
+      <c r="A35" s="10">
+        <v>46193</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" s="14">
+        <v>0</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D35" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F35" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E35" s="14">
+        <v>0</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>18</v>
@@ -2136,28 +2127,27 @@
         <v>1</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>170</v>
+        <v>108</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A36" s="7" t="s">
-        <v>120</v>
+      <c r="A36" s="10">
+        <v>46193</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" s="14">
+        <v>5</v>
+      </c>
+      <c r="D36" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D36" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F36" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>オランダ</v>
+      <c r="E36" s="14">
+        <v>1</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>8</v>
@@ -2166,28 +2156,27 @@
         <v>1</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>163</v>
+        <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A37" s="7" t="s">
-        <v>120</v>
+      <c r="A37" s="10">
+        <v>46193</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" s="14">
+        <v>0</v>
+      </c>
+      <c r="D37" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D37" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F37" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>⽇本</v>
+      <c r="E37" s="14">
+        <v>4</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>8</v>
@@ -2196,28 +2185,27 @@
         <v>1</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>165</v>
+        <v>103</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A38" s="9" t="s">
-        <v>121</v>
+      <c r="A38" s="9">
+        <v>46194</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C38" s="14">
+        <v>2</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D38" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F38" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E38" s="14">
+        <v>2</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>19</v>
@@ -2226,28 +2214,27 @@
         <v>1</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>167</v>
+        <v>105</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" s="9" t="s">
-        <v>121</v>
+      <c r="A39" s="9">
+        <v>46194</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C39" s="14">
+        <v>4</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D39" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F39" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>スペイン</v>
+      <c r="E39" s="14">
+        <v>0</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G39" s="2" t="s">
         <v>10</v>
@@ -2256,28 +2243,27 @@
         <v>1</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>166</v>
+        <v>104</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" s="9" t="s">
-        <v>121</v>
+      <c r="A40" s="9">
+        <v>46194</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" s="14">
+        <v>0</v>
+      </c>
+      <c r="D40" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D40" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F40" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E40" s="14">
+        <v>0</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>11</v>
@@ -2286,28 +2272,27 @@
         <v>1</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>157</v>
+        <v>95</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" s="9" t="s">
-        <v>121</v>
+      <c r="A41" s="9">
+        <v>46194</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C41" s="14">
+        <v>1</v>
+      </c>
+      <c r="D41" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D41" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F41" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>エジプト</v>
+      <c r="E41" s="14">
+        <v>3</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>11</v>
@@ -2316,28 +2301,27 @@
         <v>1</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>159</v>
+        <v>97</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A42" s="9" t="s">
-        <v>122</v>
+      <c r="A42" s="9">
+        <v>46195</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" s="14">
+        <v>3</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D42" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F42" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>ノルウェー</v>
+      <c r="E42" s="14">
+        <v>2</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>20</v>
@@ -2346,28 +2330,27 @@
         <v>1</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>169</v>
+        <v>107</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" s="9" t="s">
-        <v>122</v>
+      <c r="A43" s="9">
+        <v>46195</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="C43" s="14">
+        <v>3</v>
+      </c>
+      <c r="D43" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D43" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F43" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>フランス</v>
+      <c r="E43" s="14">
+        <v>0</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>13</v>
@@ -2376,28 +2359,27 @@
         <v>1</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>162</v>
+        <v>100</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A44" s="9" t="s">
-        <v>122</v>
+      <c r="A44" s="9">
+        <v>46195</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C44" s="14">
+        <v>2</v>
+      </c>
+      <c r="D44" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D44" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F44" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>アルゼンチン</v>
+      <c r="E44" s="14">
+        <v>0</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>21</v>
@@ -2406,28 +2388,27 @@
         <v>1</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>164</v>
+        <v>102</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A45" s="9" t="s">
-        <v>122</v>
+      <c r="A45" s="9">
+        <v>46195</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="C45" s="14">
+        <v>1</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D45" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F45" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>アルジェリア</v>
+      <c r="E45" s="14">
+        <v>2</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>21</v>
@@ -2436,28 +2417,27 @@
         <v>1</v>
       </c>
       <c r="I45" s="3" t="s">
-        <v>161</v>
+        <v>99</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="9" t="s">
-        <v>123</v>
+      <c r="A46" s="9">
+        <v>46196</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="C46" s="14">
+        <v>0</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D46" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F46" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E46" s="14">
+        <v>0</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>16</v>
@@ -2466,28 +2446,27 @@
         <v>1</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>158</v>
+        <v>96</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A47" s="9" t="s">
-        <v>123</v>
+      <c r="A47" s="9">
+        <v>46196</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C47" s="14">
+        <v>0</v>
+      </c>
+      <c r="D47" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D47" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F47" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>クロアチア</v>
+      <c r="E47" s="14">
+        <v>1</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G47" s="2" t="s">
         <v>16</v>
@@ -2496,28 +2475,27 @@
         <v>1</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>156</v>
+        <v>94</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A48" s="9" t="s">
-        <v>123</v>
+      <c r="A48" s="9">
+        <v>46196</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="C48" s="14">
+        <v>5</v>
+      </c>
+      <c r="D48" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D48" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F48" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>ポルトガル</v>
+      <c r="E48" s="14">
+        <v>0</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>17</v>
@@ -2526,28 +2504,27 @@
         <v>1</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>163</v>
+        <v>101</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A49" s="9" t="s">
-        <v>123</v>
+      <c r="A49" s="9">
+        <v>46196</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="C49" s="14">
+        <v>1</v>
+      </c>
+      <c r="D49" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D49" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F49" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>コロンビア</v>
+      <c r="E49" s="14">
+        <v>0</v>
+      </c>
+      <c r="F49" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>22</v>
@@ -2556,28 +2533,27 @@
         <v>1</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>155</v>
+        <v>93</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A50" s="7" t="s">
-        <v>124</v>
+      <c r="A50" s="10">
+        <v>46197</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="C50" s="14">
+        <v>0</v>
+      </c>
+      <c r="D50" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D50" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F50" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>ブラジル</v>
+      <c r="E50" s="14">
+        <v>3</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>6</v>
@@ -2586,28 +2562,27 @@
         <v>1</v>
       </c>
       <c r="I50" s="3" t="s">
-        <v>167</v>
+        <v>105</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A51" s="7" t="s">
-        <v>124</v>
+      <c r="A51" s="10">
+        <v>46197</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C51" s="1" t="s">
+      <c r="C51" s="14">
+        <v>4</v>
+      </c>
+      <c r="D51" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D51" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F51" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>モロッコ</v>
+      <c r="E51" s="14">
+        <v>2</v>
+      </c>
+      <c r="F51" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>6</v>
@@ -2616,28 +2591,27 @@
         <v>1</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>166</v>
+        <v>104</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A52" s="7" t="s">
-        <v>124</v>
+      <c r="A52" s="10">
+        <v>46197</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C52" s="1" t="s">
+      <c r="C52" s="14">
+        <v>2</v>
+      </c>
+      <c r="D52" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D52" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F52" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>スイス</v>
+      <c r="E52" s="14">
+        <v>1</v>
+      </c>
+      <c r="F52" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>2</v>
@@ -2646,28 +2620,27 @@
         <v>1</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>159</v>
+        <v>97</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A53" s="7" t="s">
-        <v>124</v>
+      <c r="A53" s="10">
+        <v>46197</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C53" s="1" t="s">
+      <c r="C53" s="14">
+        <v>3</v>
+      </c>
+      <c r="D53" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D53" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="E53" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F53" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>ボスニア・ヘルツェゴビナ</v>
+      <c r="E53" s="14">
+        <v>1</v>
+      </c>
+      <c r="F53" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>2</v>
@@ -2676,28 +2649,27 @@
         <v>1</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>168</v>
+        <v>106</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A54" s="7" t="s">
-        <v>124</v>
+      <c r="A54" s="10">
+        <v>46197</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C54" s="1" t="s">
+      <c r="C54" s="14">
+        <v>0</v>
+      </c>
+      <c r="D54" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D54" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F54" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>メキシコ</v>
+      <c r="E54" s="14">
+        <v>3</v>
+      </c>
+      <c r="F54" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G54" s="2" t="s">
         <v>0</v>
@@ -2706,28 +2678,27 @@
         <v>1</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>154</v>
+        <v>92</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A55" s="7" t="s">
-        <v>124</v>
+      <c r="A55" s="10">
+        <v>46197</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C55" s="1" t="s">
+      <c r="C55" s="14">
+        <v>1</v>
+      </c>
+      <c r="D55" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D55" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F55" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>南アフリカ</v>
+      <c r="E55" s="14">
+        <v>0</v>
+      </c>
+      <c r="F55" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>0</v>
@@ -2736,28 +2707,27 @@
         <v>1</v>
       </c>
       <c r="I55" s="3" t="s">
-        <v>165</v>
+        <v>103</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A56" s="9" t="s">
-        <v>125</v>
+      <c r="A56" s="9">
+        <v>46198</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="C56" s="14">
+        <v>0</v>
+      </c>
+      <c r="D56" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D56" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F56" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>コートジボワール</v>
+      <c r="E56" s="14">
+        <v>2</v>
+      </c>
+      <c r="F56" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>7</v>
@@ -2766,28 +2736,27 @@
         <v>1</v>
       </c>
       <c r="I56" s="3" t="s">
-        <v>162</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A57" s="9" t="s">
-        <v>125</v>
+      <c r="A57" s="9">
+        <v>46198</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C57" s="1" t="s">
+      <c r="C57" s="14">
+        <v>2</v>
+      </c>
+      <c r="D57" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D57" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="E57" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F57" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>エクアドル</v>
+      <c r="E57" s="14">
+        <v>1</v>
+      </c>
+      <c r="F57" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>7</v>
@@ -2796,28 +2765,27 @@
         <v>1</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>169</v>
+        <v>107</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A58" s="9" t="s">
-        <v>125</v>
+      <c r="A58" s="9">
+        <v>46198</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C58" s="1" t="s">
+      <c r="C58" s="14">
+        <v>1</v>
+      </c>
+      <c r="D58" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D58" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F58" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E58" s="14">
+        <v>1</v>
+      </c>
+      <c r="F58" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>8</v>
@@ -2826,28 +2794,27 @@
         <v>1</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>164</v>
+        <v>102</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A59" s="9" t="s">
-        <v>125</v>
+      <c r="A59" s="9">
+        <v>46198</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C59" s="1" t="s">
+      <c r="C59" s="14">
+        <v>1</v>
+      </c>
+      <c r="D59" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D59" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="E59" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F59" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>オランダ</v>
+      <c r="E59" s="14">
+        <v>3</v>
+      </c>
+      <c r="F59" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>8</v>
@@ -2856,28 +2823,27 @@
         <v>1</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>170</v>
+        <v>108</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A60" s="9" t="s">
-        <v>125</v>
+      <c r="A60" s="9">
+        <v>46198</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C60" s="1" t="s">
+      <c r="C60" s="14">
+        <v>3</v>
+      </c>
+      <c r="D60" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D60" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E60" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F60" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>トルコ</v>
+      <c r="E60" s="14">
+        <v>2</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>3</v>
@@ -2886,28 +2852,27 @@
         <v>1</v>
       </c>
       <c r="I60" s="3" t="s">
-        <v>157</v>
+        <v>95</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A61" s="9" t="s">
-        <v>125</v>
+      <c r="A61" s="9">
+        <v>46198</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C61" s="1" t="s">
+      <c r="C61" s="14">
+        <v>0</v>
+      </c>
+      <c r="D61" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D61" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="E61" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F61" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E61" s="14">
+        <v>0</v>
+      </c>
+      <c r="F61" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>23</v>
@@ -2916,28 +2881,27 @@
         <v>1</v>
       </c>
       <c r="I61" s="3" t="s">
-        <v>161</v>
+        <v>99</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A62" s="9" t="s">
-        <v>126</v>
+      <c r="A62" s="9">
+        <v>46199</v>
       </c>
       <c r="B62" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C62" s="1" t="s">
+      <c r="C62" s="14">
+        <v>1</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D62" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="E62" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F62" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>フランス</v>
+      <c r="E62" s="14">
+        <v>4</v>
+      </c>
+      <c r="F62" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G62" s="2" t="s">
         <v>20</v>
@@ -2946,28 +2910,27 @@
         <v>1</v>
       </c>
       <c r="I62" s="3" t="s">
-        <v>158</v>
+        <v>96</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A63" s="9" t="s">
-        <v>126</v>
+      <c r="A63" s="9">
+        <v>46199</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C63" s="1" t="s">
+      <c r="C63" s="14">
+        <v>5</v>
+      </c>
+      <c r="D63" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D63" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="E63" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F63" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>セネガル</v>
+      <c r="E63" s="14">
+        <v>0</v>
+      </c>
+      <c r="F63" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G63" s="2" t="s">
         <v>13</v>
@@ -2976,28 +2939,27 @@
         <v>1</v>
       </c>
       <c r="I63" s="3" t="s">
-        <v>156</v>
+        <v>94</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A64" s="9" t="s">
-        <v>126</v>
+      <c r="A64" s="9">
+        <v>46199</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C64" s="1" t="s">
+      <c r="C64" s="14">
+        <v>1</v>
+      </c>
+      <c r="D64" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D64" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E64" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F64" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E64" s="14">
+        <v>1</v>
+      </c>
+      <c r="F64" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G64" s="2" t="s">
         <v>11</v>
@@ -3006,28 +2968,27 @@
         <v>1</v>
       </c>
       <c r="I64" s="3" t="s">
-        <v>168</v>
+        <v>106</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A65" s="9" t="s">
-        <v>126</v>
+      <c r="A65" s="9">
+        <v>46199</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C65" s="1" t="s">
+      <c r="C65" s="14">
+        <v>1</v>
+      </c>
+      <c r="D65" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D65" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="E65" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F65" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>ベルギー</v>
+      <c r="E65" s="14">
+        <v>5</v>
+      </c>
+      <c r="F65" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G65" s="2" t="s">
         <v>11</v>
@@ -3036,28 +2997,27 @@
         <v>1</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>159</v>
+        <v>97</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A66" s="9" t="s">
-        <v>126</v>
+      <c r="A66" s="9">
+        <v>46199</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C66" s="1" t="s">
+      <c r="C66" s="14">
+        <v>0</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D66" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="E66" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F66" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>引き分け</v>
+      <c r="E66" s="14">
+        <v>0</v>
+      </c>
+      <c r="F66" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G66" s="2" t="s">
         <v>10</v>
@@ -3066,28 +3026,27 @@
         <v>1</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>163</v>
+        <v>101</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A67" s="9" t="s">
-        <v>126</v>
+      <c r="A67" s="9">
+        <v>46199</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C67" s="1" t="s">
+      <c r="C67" s="14">
+        <v>0</v>
+      </c>
+      <c r="D67" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D67" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E67" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F67" s="6" t="str">
-        <f t="shared" ref="F67:F105" si="1">_xlfn.LET(_xlpm.s,D67,_xlpm.hs,--_xlfn.TEXTBEFORE(_xlpm.s,"-"),_xlpm.as,--_xlfn.TEXTAFTER(_xlpm.s,"-"),IF(_xlpm.hs&gt;_xlpm.as,B67,IF(_xlpm.hs&lt;_xlpm.as,C67,"引き分け")))</f>
-        <v>スペイン</v>
+      <c r="E67" s="14">
+        <v>1</v>
+      </c>
+      <c r="F67" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G67" s="2" t="s">
         <v>10</v>
@@ -3096,28 +3055,27 @@
         <v>1</v>
       </c>
       <c r="I67" s="3" t="s">
-        <v>155</v>
+        <v>93</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A68" s="9" t="s">
-        <v>127</v>
+      <c r="A68" s="9">
+        <v>46200</v>
       </c>
       <c r="B68" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C68" s="1" t="s">
+      <c r="C68" s="14">
+        <v>0</v>
+      </c>
+      <c r="D68" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D68" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="E68" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F68" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>イングランド</v>
+      <c r="E68" s="14">
+        <v>2</v>
+      </c>
+      <c r="F68" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G68" s="2" t="s">
         <v>24</v>
@@ -3126,28 +3084,27 @@
         <v>1</v>
       </c>
       <c r="I68" s="3" t="s">
-        <v>169</v>
+        <v>107</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A69" s="9" t="s">
-        <v>127</v>
+      <c r="A69" s="9">
+        <v>46200</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C69" s="1" t="s">
+      <c r="C69" s="14">
+        <v>2</v>
+      </c>
+      <c r="D69" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D69" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="E69" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F69" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>クロアチア</v>
+      <c r="E69" s="14">
+        <v>1</v>
+      </c>
+      <c r="F69" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G69" s="2" t="s">
         <v>24</v>
@@ -3156,28 +3113,27 @@
         <v>1</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>162</v>
+        <v>100</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A70" s="9" t="s">
-        <v>127</v>
+      <c r="A70" s="9">
+        <v>46200</v>
       </c>
       <c r="B70" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C70" s="1" t="s">
+      <c r="C70" s="14">
+        <v>3</v>
+      </c>
+      <c r="D70" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D70" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="E70" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F70" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>引き分け</v>
+      <c r="E70" s="14">
+        <v>3</v>
+      </c>
+      <c r="F70" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G70" s="2" t="s">
         <v>21</v>
@@ -3186,28 +3142,27 @@
         <v>1</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>170</v>
+        <v>108</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A71" s="9" t="s">
-        <v>127</v>
+      <c r="A71" s="9">
+        <v>46200</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C71" s="1" t="s">
+      <c r="C71" s="14">
+        <v>1</v>
+      </c>
+      <c r="D71" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D71" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="E71" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F71" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>アルゼンチン</v>
+      <c r="E71" s="14">
+        <v>3</v>
+      </c>
+      <c r="F71" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G71" s="2" t="s">
         <v>21</v>
@@ -3216,28 +3171,27 @@
         <v>1</v>
       </c>
       <c r="I71" s="3" t="s">
-        <v>164</v>
+        <v>102</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A72" s="9" t="s">
-        <v>127</v>
+      <c r="A72" s="9">
+        <v>46200</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C72" s="1" t="s">
+      <c r="C72" s="14">
+        <v>0</v>
+      </c>
+      <c r="D72" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D72" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="E72" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F72" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>引き分け</v>
+      <c r="E72" s="14">
+        <v>0</v>
+      </c>
+      <c r="F72" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G72" s="2" t="s">
         <v>17</v>
@@ -3246,28 +3200,27 @@
         <v>1</v>
       </c>
       <c r="I72" s="3" t="s">
-        <v>167</v>
+        <v>105</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A73" s="9" t="s">
-        <v>127</v>
+      <c r="A73" s="9">
+        <v>46200</v>
       </c>
       <c r="B73" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C73" s="1" t="s">
+      <c r="C73" s="14">
+        <v>3</v>
+      </c>
+      <c r="D73" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D73" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="E73" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F73" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>コンゴ⺠主共和国</v>
+      <c r="E73" s="14">
+        <v>1</v>
+      </c>
+      <c r="F73" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="G73" s="2" t="s">
         <v>17</v>
@@ -3276,875 +3229,844 @@
         <v>1</v>
       </c>
       <c r="I73" s="3" t="s">
-        <v>166</v>
+        <v>104</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A74" s="9" t="s">
-        <v>128</v>
+      <c r="A74" s="9">
+        <v>46201</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C74" s="1" t="s">
+      <c r="C74" s="14">
+        <v>0</v>
+      </c>
+      <c r="D74" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D74" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E74" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F74" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>カナダ</v>
+      <c r="E74" s="14">
+        <v>1</v>
+      </c>
+      <c r="F74" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H74" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I74" s="3" t="s">
-        <v>171</v>
+        <v>109</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A75" s="9" t="s">
-        <v>129</v>
+      <c r="A75" s="9">
+        <v>46202</v>
       </c>
       <c r="B75" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C75" s="1" t="s">
+      <c r="C75" s="14">
+        <v>1</v>
+      </c>
+      <c r="D75" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D75" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E75" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="F75" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>引き分け</v>
+      <c r="E75" s="14">
+        <v>1</v>
+      </c>
+      <c r="F75" s="5" t="s">
+        <v>79</v>
       </c>
       <c r="H75" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I75" s="3" t="s">
-        <v>158</v>
+        <v>96</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A76" s="9" t="s">
-        <v>129</v>
+      <c r="A76" s="9">
+        <v>46202</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C76" s="1" t="s">
+      <c r="C76" s="14">
+        <v>1</v>
+      </c>
+      <c r="D76" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D76" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E76" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F76" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>引き分け</v>
+      <c r="E76" s="14">
+        <v>1</v>
+      </c>
+      <c r="F76" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="H76" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>165</v>
+        <v>103</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A77" s="9" t="s">
-        <v>129</v>
+      <c r="A77" s="9">
+        <v>46202</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C77" s="2" t="s">
+      <c r="C77" s="15">
+        <v>2</v>
+      </c>
+      <c r="D77" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D77" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="E77" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="F77" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>ブラジル</v>
+      <c r="E77" s="15">
+        <v>1</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>84</v>
       </c>
       <c r="H77" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I77" s="3" t="s">
-        <v>163</v>
+        <v>101</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A78" s="9" t="s">
-        <v>130</v>
+      <c r="A78" s="9">
+        <v>46203</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C78" s="1" t="s">
+      <c r="C78" s="14">
+        <v>3</v>
+      </c>
+      <c r="D78" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D78" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E78" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F78" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>フランス</v>
+      <c r="E78" s="14">
+        <v>0</v>
+      </c>
+      <c r="F78" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H78" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I78" s="3" t="s">
-        <v>169</v>
+        <v>107</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A79" s="9" t="s">
-        <v>130</v>
+      <c r="A79" s="9">
+        <v>46203</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C79" s="1" t="s">
+      <c r="C79" s="14">
+        <v>1</v>
+      </c>
+      <c r="D79" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D79" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="E79" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F79" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>ノルウェー</v>
+      <c r="E79" s="14">
+        <v>2</v>
+      </c>
+      <c r="F79" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H79" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I79" s="3" t="s">
-        <v>164</v>
+        <v>102</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A80" s="9" t="s">
-        <v>130</v>
+      <c r="A80" s="9">
+        <v>46203</v>
       </c>
       <c r="B80" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C80" s="1" t="s">
+      <c r="C80" s="14">
+        <v>2</v>
+      </c>
+      <c r="D80" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D80" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E80" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F80" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>メキシコ</v>
+      <c r="E80" s="14">
+        <v>0</v>
+      </c>
+      <c r="F80" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H80" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I80" s="3" t="s">
-        <v>154</v>
+        <v>92</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A81" s="7" t="s">
-        <v>131</v>
+      <c r="A81" s="10">
+        <v>46204</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C81" s="1" t="s">
+      <c r="C81" s="14">
+        <v>2</v>
+      </c>
+      <c r="D81" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D81" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="E81" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F81" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>イングランド</v>
+      <c r="E81" s="14">
+        <v>1</v>
+      </c>
+      <c r="F81" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H81" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I81" s="3" t="s">
-        <v>166</v>
+        <v>104</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A82" s="7" t="s">
-        <v>131</v>
+      <c r="A82" s="10">
+        <v>46204</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C82" s="1" t="s">
+      <c r="C82" s="14">
+        <v>2</v>
+      </c>
+      <c r="D82" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D82" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E82" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F82" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>アメリカ</v>
+      <c r="E82" s="14">
+        <v>0</v>
+      </c>
+      <c r="F82" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H82" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I82" s="3" t="s">
-        <v>161</v>
+        <v>99</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A83" s="7" t="s">
-        <v>131</v>
+      <c r="A83" s="10">
+        <v>46204</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C83" s="1" t="s">
+      <c r="C83" s="14">
+        <v>3</v>
+      </c>
+      <c r="D83" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D83" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E83" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F83" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>ベルギー</v>
+      <c r="E83" s="14">
+        <v>2</v>
+      </c>
+      <c r="F83" s="5" t="s">
+        <v>81</v>
       </c>
       <c r="H83" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I83" s="3" t="s">
-        <v>168</v>
+        <v>106</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A84" s="9" t="s">
-        <v>132</v>
+      <c r="A84" s="9">
+        <v>46205</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C84" s="1" t="s">
+      <c r="C84" s="14">
+        <v>2</v>
+      </c>
+      <c r="D84" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D84" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="E84" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F84" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>ポルトガル</v>
+      <c r="E84" s="14">
+        <v>1</v>
+      </c>
+      <c r="F84" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H84" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I84" s="3" t="s">
-        <v>156</v>
+        <v>94</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A85" s="9" t="s">
-        <v>132</v>
+      <c r="A85" s="9">
+        <v>46205</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C85" s="1" t="s">
+      <c r="C85" s="14">
+        <v>3</v>
+      </c>
+      <c r="D85" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D85" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E85" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F85" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>スペイン</v>
+      <c r="E85" s="14">
+        <v>0</v>
+      </c>
+      <c r="F85" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H85" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I85" s="3" t="s">
-        <v>157</v>
+        <v>95</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A86" s="9" t="s">
-        <v>132</v>
+      <c r="A86" s="9">
+        <v>46205</v>
       </c>
       <c r="B86" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C86" s="1" t="s">
+      <c r="C86" s="14">
+        <v>2</v>
+      </c>
+      <c r="D86" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D86" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E86" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F86" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>スイス</v>
+      <c r="E86" s="14">
+        <v>0</v>
+      </c>
+      <c r="F86" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H86" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>159</v>
+        <v>97</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A87" s="9" t="s">
-        <v>133</v>
+      <c r="A87" s="9">
+        <v>46206</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C87" s="1" t="s">
+      <c r="C87" s="14">
+        <v>3</v>
+      </c>
+      <c r="D87" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D87" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E87" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F87" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>アルゼンチン</v>
+      <c r="E87" s="14">
+        <v>2</v>
+      </c>
+      <c r="F87" s="5" t="s">
+        <v>81</v>
       </c>
       <c r="H87" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I87" s="3" t="s">
-        <v>167</v>
+        <v>105</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A88" s="9" t="s">
-        <v>133</v>
+      <c r="A88" s="9">
+        <v>46206</v>
       </c>
       <c r="B88" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C88" s="1" t="s">
+      <c r="C88" s="14">
+        <v>1</v>
+      </c>
+      <c r="D88" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D88" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E88" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F88" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>コロンビア</v>
+      <c r="E88" s="14">
+        <v>0</v>
+      </c>
+      <c r="F88" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H88" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>170</v>
+        <v>108</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A89" s="9" t="s">
-        <v>133</v>
+      <c r="A89" s="9">
+        <v>46206</v>
       </c>
       <c r="B89" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C89" s="1" t="s">
+      <c r="C89" s="14">
+        <v>1</v>
+      </c>
+      <c r="D89" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D89" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E89" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="F89" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>引き分け</v>
+      <c r="E89" s="14">
+        <v>1</v>
+      </c>
+      <c r="F89" s="5" t="s">
+        <v>82</v>
       </c>
       <c r="H89" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I89" s="3" t="s">
-        <v>164</v>
+        <v>102</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A90" s="9" t="s">
-        <v>134</v>
+      <c r="A90" s="9">
+        <v>46207</v>
       </c>
       <c r="B90" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C90" s="1" t="s">
+      <c r="C90" s="14">
+        <v>0</v>
+      </c>
+      <c r="D90" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="D90" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E90" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F90" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>フランス</v>
+      <c r="E90" s="14">
+        <v>1</v>
+      </c>
+      <c r="F90" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H90" s="2" t="s">
         <v>26</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>162</v>
+        <v>100</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A91" s="9" t="s">
-        <v>134</v>
+      <c r="A91" s="9">
+        <v>46207</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C91" s="1" t="s">
+      <c r="C91" s="14">
+        <v>0</v>
+      </c>
+      <c r="D91" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D91" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="E91" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F91" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>モロッコ</v>
+      <c r="E91" s="14">
+        <v>3</v>
+      </c>
+      <c r="F91" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H91" s="2" t="s">
         <v>26</v>
       </c>
       <c r="I91" s="3" t="s">
-        <v>163</v>
+        <v>101</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A92" s="9" t="s">
-        <v>135</v>
+      <c r="A92" s="9">
+        <v>46208</v>
       </c>
       <c r="B92" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C92" s="1" t="s">
+      <c r="C92" s="14">
+        <v>1</v>
+      </c>
+      <c r="D92" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D92" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="E92" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F92" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>ノルウェー</v>
+      <c r="E92" s="14">
+        <v>2</v>
+      </c>
+      <c r="F92" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H92" s="2" t="s">
         <v>26</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>169</v>
+        <v>107</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A93" s="9" t="s">
-        <v>135</v>
+      <c r="A93" s="9">
+        <v>46208</v>
       </c>
       <c r="B93" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C93" s="1" t="s">
+      <c r="C93" s="14">
+        <v>2</v>
+      </c>
+      <c r="D93" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D93" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="E93" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F93" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>イングランド</v>
+      <c r="E93" s="14">
+        <v>3</v>
+      </c>
+      <c r="F93" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H93" s="2" t="s">
         <v>26</v>
       </c>
       <c r="I93" s="3" t="s">
-        <v>154</v>
+        <v>92</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A94" s="9" t="s">
-        <v>136</v>
+      <c r="A94" s="9">
+        <v>46209</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C94" s="1" t="s">
+      <c r="C94" s="14">
+        <v>0</v>
+      </c>
+      <c r="D94" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D94" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E94" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F94" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>スペイン</v>
+      <c r="E94" s="14">
+        <v>1</v>
+      </c>
+      <c r="F94" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H94" s="2" t="s">
         <v>26</v>
       </c>
       <c r="I94" s="3" t="s">
-        <v>164</v>
+        <v>102</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A95" s="9" t="s">
-        <v>136</v>
+      <c r="A95" s="9">
+        <v>46209</v>
       </c>
       <c r="B95" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C95" s="1" t="s">
+      <c r="C95" s="14">
+        <v>1</v>
+      </c>
+      <c r="D95" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D95" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="E95" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F95" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>ベルギー</v>
+      <c r="E95" s="14">
+        <v>3</v>
+      </c>
+      <c r="F95" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H95" s="2" t="s">
         <v>26</v>
       </c>
       <c r="I95" s="3" t="s">
-        <v>168</v>
+        <v>106</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A96" s="9" t="s">
-        <v>137</v>
+      <c r="A96" s="9">
+        <v>46210</v>
       </c>
       <c r="B96" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C96" s="1" t="s">
+      <c r="C96" s="14">
+        <v>3</v>
+      </c>
+      <c r="D96" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D96" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E96" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F96" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>アルゼンチン</v>
+      <c r="E96" s="14">
+        <v>2</v>
+      </c>
+      <c r="F96" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H96" s="2" t="s">
         <v>26</v>
       </c>
       <c r="I96" s="3" t="s">
-        <v>166</v>
+        <v>104</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A97" s="9" t="s">
-        <v>137</v>
+      <c r="A97" s="9">
+        <v>46210</v>
       </c>
       <c r="B97" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C97" s="1" t="s">
+      <c r="C97" s="14">
+        <v>0</v>
+      </c>
+      <c r="D97" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D97" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="E97" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="F97" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>引き分け</v>
+      <c r="E97" s="14">
+        <v>0</v>
+      </c>
+      <c r="F97" s="5" t="s">
+        <v>83</v>
       </c>
       <c r="H97" s="2" t="s">
         <v>26</v>
       </c>
       <c r="I97" s="3" t="s">
-        <v>159</v>
+        <v>97</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A98" s="9" t="s">
-        <v>138</v>
+      <c r="A98" s="9">
+        <v>46212</v>
       </c>
       <c r="B98" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C98" s="1" t="s">
+      <c r="C98" s="14">
+        <v>2</v>
+      </c>
+      <c r="D98" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D98" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E98" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F98" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>フランス</v>
+      <c r="E98" s="14">
+        <v>0</v>
+      </c>
+      <c r="F98" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H98" s="2" t="s">
         <v>27</v>
       </c>
       <c r="I98" s="3" t="s">
-        <v>158</v>
+        <v>96</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A99" s="9" t="s">
-        <v>139</v>
+      <c r="A99" s="9">
+        <v>46213</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C99" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D99" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E99" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F99" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>フランス</v>
-      </c>
+        <v>112</v>
+      </c>
+      <c r="C99" s="14">
+        <v>2</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E99" s="14">
+        <v>1</v>
+      </c>
+      <c r="F99" s="5"/>
       <c r="H99" s="2" t="s">
         <v>27</v>
       </c>
       <c r="I99" s="3" t="s">
-        <v>157</v>
+        <v>95</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A100" s="9" t="s">
-        <v>140</v>
+      <c r="A100" s="9">
+        <v>46214</v>
       </c>
       <c r="B100" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C100" s="1" t="s">
+      <c r="C100" s="14">
+        <v>1</v>
+      </c>
+      <c r="D100" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D100" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="E100" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F100" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>イングランド</v>
+      <c r="E100" s="14">
+        <v>2</v>
+      </c>
+      <c r="F100" s="5" t="s">
+        <v>81</v>
       </c>
       <c r="H100" s="2" t="s">
         <v>27</v>
       </c>
       <c r="I100" s="3" t="s">
-        <v>167</v>
+        <v>105</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A101" s="9" t="s">
-        <v>140</v>
+      <c r="A101" s="9">
+        <v>46214</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C101" s="1" t="s">
+      <c r="C101" s="14">
+        <v>3</v>
+      </c>
+      <c r="D101" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D101" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="E101" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F101" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>アルゼンチン</v>
+      <c r="E101" s="14">
+        <v>1</v>
+      </c>
+      <c r="F101" s="5" t="s">
+        <v>81</v>
       </c>
       <c r="H101" s="2" t="s">
         <v>27</v>
       </c>
       <c r="I101" s="3" t="s">
-        <v>170</v>
+        <v>108</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A102" s="7" t="s">
-        <v>141</v>
+      <c r="A102" s="10">
+        <v>46217</v>
       </c>
       <c r="B102" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C102" s="4" t="s">
+      <c r="C102" s="16">
+        <v>0</v>
+      </c>
+      <c r="D102" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D102" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E102" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="F102" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v>スペイン</v>
+      <c r="E102" s="16">
+        <v>2</v>
+      </c>
+      <c r="F102" s="7" t="s">
+        <v>84</v>
       </c>
       <c r="H102" s="3" t="s">
         <v>28</v>
       </c>
       <c r="I102" s="3" t="s">
-        <v>164</v>
+        <v>102</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A103" s="9" t="s">
-        <v>142</v>
+      <c r="A103" s="9">
+        <v>46218</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C103" s="1" t="s">
+      <c r="C103" s="14">
+        <v>1</v>
+      </c>
+      <c r="D103" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D103" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="E103" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F103" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>アルゼンチン</v>
+      <c r="E103" s="14">
+        <v>2</v>
+      </c>
+      <c r="F103" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H103" s="3" t="s">
         <v>28</v>
       </c>
       <c r="I103" s="3" t="s">
-        <v>166</v>
+        <v>104</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A104" s="9" t="s">
-        <v>143</v>
+      <c r="A104" s="9">
+        <v>46221</v>
       </c>
       <c r="B104" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C104" s="1" t="s">
+      <c r="C104" s="14">
+        <v>4</v>
+      </c>
+      <c r="D104" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D104" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="E104" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F104" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>イングランド</v>
+      <c r="E104" s="14">
+        <v>6</v>
+      </c>
+      <c r="F104" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="H104" s="2" t="s">
         <v>29</v>
       </c>
       <c r="I104" s="3" t="s">
-        <v>167</v>
+        <v>105</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A105" s="9" t="s">
-        <v>144</v>
+      <c r="A105" s="9">
+        <v>46222</v>
       </c>
       <c r="B105" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C105" s="1" t="s">
+      <c r="C105" s="14">
+        <v>1</v>
+      </c>
+      <c r="D105" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D105" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E105" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F105" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>スペイン</v>
+      <c r="E105" s="14">
+        <v>0</v>
+      </c>
+      <c r="F105" s="5" t="s">
+        <v>81</v>
       </c>
       <c r="H105" s="2" t="s">
         <v>30</v>
       </c>
       <c r="I105" s="3" t="s">
-        <v>169</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>